<commit_message>
fix timezone + add forgot checkout mail service
</commit_message>
<xml_diff>
--- a/src/main/resources/input/cham-cong.xlsx
+++ b/src/main/resources/input/cham-cong.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\KITS\Project\code\attendance-tool\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\attendance-tool\src\main\resources\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E18931B-9613-491E-A5B9-0CB538EB28CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{661961D9-17ED-4655-916C-849D71C99EE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="47">
   <si>
     <t>ID</t>
   </si>
@@ -155,6 +155,12 @@
   </si>
   <si>
     <t>emp19@xyz.com</t>
+  </si>
+  <si>
+    <t>Mr 67</t>
+  </si>
+  <si>
+    <t>phuc02032004@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -165,7 +171,7 @@
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
     <numFmt numFmtId="165" formatCode="h:mm:ss;@"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -189,6 +195,14 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -223,10 +237,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -248,8 +263,10 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -550,13 +567,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6" style="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.33203125" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.44140625" style="5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8" style="3" customWidth="1"/>
     <col min="6" max="6" width="8.109375" style="2" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.5546875" style="1" bestFit="1" customWidth="1"/>
@@ -1629,9 +1646,65 @@
         <v>0.99930555555555556</v>
       </c>
     </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A42" s="4">
+        <v>93041</v>
+      </c>
+      <c r="B42" s="4">
+        <v>67</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D42" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="E42" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F42" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G42" s="1">
+        <v>45987</v>
+      </c>
+      <c r="H42" s="9">
+        <v>0.43055555555555558</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A43" s="4">
+        <v>93042</v>
+      </c>
+      <c r="B43" s="4">
+        <v>67</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D43" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="E43" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F43" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G43" s="1">
+        <v>45987</v>
+      </c>
+      <c r="H43" s="9">
+        <v>0.99930555555555556</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="D42" r:id="rId1" xr:uid="{71F1E0DF-706A-41E0-A1DC-14E44ED0D48C}"/>
+    <hyperlink ref="D43" r:id="rId2" xr:uid="{44B2BAD9-175D-46A4-814B-5A81247432A0}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>